<commit_message>
-binding redirect de Microsoft.Bcl.Memory a 9.0.0.0 -restaurar Swashbuckle/WebActivatorEx en csproj + binding redirect Bcl.Memory (Swagger)
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios de aceptación" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definition of Done" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sprint" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Historias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tareas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Criterios de aceptación" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Definition of Done" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Historias'!$A$5:$P$29</definedName>
@@ -514,51 +514,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1257120</colOff>
-      <row>3</row>
-      <rowOff>37440</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="211320" y="190440"/>
-          <a:ext cx="1257120" cy="418680"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1169,7 +1124,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1639,7 +1593,7 @@
       </c>
       <c r="N10" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr">
@@ -1647,7 +1601,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P10" s="12" t="n"/>
+      <c r="P10" s="17" t="inlineStr">
+        <is>
+          <t>Construida por Emilio Fuentes (11-09-2026) siguiendo PATRONES/ASP: BD SEL/INS/UPD/DEL_CHECKLIST_PLANTILLA (patron dinamico, FNC_PAIS_HORA, INS_EXCEPCION, codigo unico por cliente, baja logica) + estructura Version/Seccion/Item/Validacion (BD/192) + lookups (BD/189,191,194). Web: ChecklistPlantillas/ChecklistPlantilla/ChecklistPlantillaVista con Model+Controllers; editor inline de secciones y campos; previsualizacion de solo lectura al clic. Datos reales: SOP-09-R24 con 25 secciones y 208 campos (BD/193). Seguridad por cliente + Token + Menu_Funcion. Compila exitcode=0 y SP probados en transaccion revertida. PENDIENTE (otra persona): pruebas por criterio, documentacion y consumo movil.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="69" customHeight="1" s="19">
       <c r="A11" s="13" t="inlineStr">
@@ -3112,6 +3070,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="19">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -5426,11 +5386,15 @@
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I59" s="11" t="n"/>
-      <c r="J59" s="12" t="n"/>
+      <c r="J59" s="17" t="inlineStr">
+        <is>
+          <t>Revisado Checklist_Plantilla (cols/FK); confirmado el unico UX_CPL_CLIENTE_CODIGO (cpl_cliente,cpl_codigo), garantizado idempotente. BD/189.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="27.6" customHeight="1" s="19">
       <c r="A60" s="11" t="inlineStr">
@@ -5468,11 +5432,15 @@
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I60" s="11" t="n"/>
-      <c r="J60" s="12" t="n"/>
+      <c r="J60" s="17" t="inlineStr">
+        <is>
+          <t>SEL_CHECKLIST_PLANTILLA: patron dinamico @SELECT/@FROM/@WHERE, @FILTRO escapado, auditoria con nombre de usuario (LEFT JOIN Usuario), ORDER BY cpl_codigo. Un solo SP grilla+ficha+combos. BD/189.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="27.6" customHeight="1" s="19">
       <c r="A61" s="11" t="inlineStr">
@@ -5510,11 +5478,15 @@
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I61" s="11" t="n"/>
-      <c r="J61" s="12" t="n"/>
+      <c r="J61" s="17" t="inlineStr">
+        <is>
+          <t>INS_CHECKLIST_PLANTILLA: alta en transaccion, codigo unico por cliente, planta del mismo cliente, sella fecha con FNC_PAIS_HORA, INS_EXCEPCION. BD/189.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="41.4" customHeight="1" s="19">
       <c r="A62" s="11" t="inlineStr">
@@ -5552,11 +5524,15 @@
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I62" s="11" t="n"/>
-      <c r="J62" s="12" t="n"/>
+      <c r="J62" s="17" t="inlineStr">
+        <is>
+          <t>UPD_CHECKLIST_PLANTILLA: @ID/@USUARIO obligatorios; ISNULL(@X,col) en codigo/nombre/habilitado; codigo unico excluyendo el propio. BD/189.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="27.6" customHeight="1" s="19">
       <c r="A63" s="11" t="inlineStr">
@@ -5594,11 +5570,15 @@
       </c>
       <c r="H63" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I63" s="11" t="n"/>
-      <c r="J63" s="12" t="n"/>
+      <c r="J63" s="17" t="inlineStr">
+        <is>
+          <t>DEL_CHECKLIST_PLANTILLA: baja logica (cpl_habilitado=0); rechaza si tiene versiones PUBLICADAS (un borrador no bloquea). BD/189.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="27.6" customHeight="1" s="19">
       <c r="A64" s="11" t="inlineStr">
@@ -5636,11 +5616,15 @@
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I64" s="11" t="n"/>
-      <c r="J64" s="12" t="n"/>
+      <c r="J64" s="17" t="inlineStr">
+        <is>
+          <t>Datos de prueba: pauta real SOP-09-R24 (Check List Servicios, Hamburgo) con 25 secciones y 208 campos via los SP; se deshabilito el checklist demo de la App. BD/190 y BD/193.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="27.6" customHeight="1" s="19">
       <c r="A65" s="11" t="inlineStr">
@@ -5678,11 +5662,15 @@
       </c>
       <c r="H65" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I65" s="11" t="n"/>
-      <c r="J65" s="12" t="n"/>
+      <c r="J65" s="17" t="inlineStr">
+        <is>
+          <t>ChecklistPlantillas.aspx: grilla RadGrid2 + wucFiltro (busqueda + habilitados) + Nuevo/Dar de baja; clic en fila = previsualizacion de solo lectura.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="27.6" customHeight="1" s="19">
       <c r="A66" s="11" t="inlineStr">
@@ -5720,11 +5708,15 @@
       </c>
       <c r="H66" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I66" s="11" t="n"/>
-      <c r="J66" s="12" t="n"/>
+      <c r="J66" s="17" t="inlineStr">
+        <is>
+          <t>ChecklistPlantilla.aspx (RadWindow, sigma-modal-* seccionada: Identificacion, Alcance y Campos del checklist); combos por SEL_; CustomValidator+validaControl; wuc:Auditoria; editor inline de secciones+campos (BD/192).</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="27.6" customHeight="1" s="19">
       <c r="A67" s="11" t="inlineStr">
@@ -5762,11 +5754,15 @@
       </c>
       <c r="H67" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I67" s="11" t="n"/>
-      <c r="J67" s="12" t="n"/>
+      <c r="J67" s="17" t="inlineStr">
+        <is>
+          <t>Menus (BD/191 y BD/194): listado + ficha + vista bajo Mantenimiento; permisos VER PAUTAS / CREAR EDITAR PAUTAS + Menu_Funcion + Perfil_Permiso.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="55.2" customHeight="1" s="19">
       <c r="A68" s="11" t="inlineStr">
@@ -5804,11 +5800,15 @@
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I68" s="11" t="n"/>
-      <c r="J68" s="12" t="n"/>
+      <c r="J68" s="17" t="inlineStr">
+        <is>
+          <t>Seguridad en servidor: listado filtra por Session.ClienteId(); Token.PuedeFuncion en la barra y Token.Puede("CREAR EDITAR PAUTAS") en la ficha; el SP filtra por cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="41.4" customHeight="1" s="19">
       <c r="A69" s="11" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="G69" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="H69" s="11" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="G70" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="G71" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Emilio Fuentes</t>
         </is>
       </c>
       <c r="H71" s="11" t="inlineStr">

</xml_diff>